<commit_message>
Restore unentered September mail and record the PDF QC.
Hold rows with no bill, and skips that were not a real statement, credit, past-due notice, POD, or payment, are back in the Inbox under AI Needs Review. The QC sheet compares each created bill to the printed invoice. No KIMCO writes.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-sept-catchup-2026-10-06.xlsx
+++ b/runs/AP-sept-catchup-2026-10-06.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="September catch-up" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="QC" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'September catch-up'!$A$1:$K$621</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QC'!$A$1:$H$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22492,4 +22494,1455 @@
   <autoFilter ref="A1:K621"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Bill id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Invoice #</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PDF total</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Live verification</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Live invoice amount</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>10465</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1086-HUDSON ENERGY-24312</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2609000773</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2448.46</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2448.46</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3302.09</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>PDF amount due $2,448.46 matches verification. Printed charges include energy $1,300.03, TDSP $900.88, securitization $0.42 and $12.12, ERCOT admin $1.42, and taxes $11.03 + $137.90 + $11.03 + $22.06. KIMCO has no merchandise lines and no Taxes tab. Fees are $2,387.25 (the PDF payment/adjustment total, saved as a positive fee), $900.88, $0.42, $12.12, and $1.42, so Invoice_Amount is $3,302.09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>10466</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1182-TRACE METAL INDUSTRIES, INC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>237704</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>165.2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>165.2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>165.2</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>10468</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1381-TRICOR METALS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>000444279/1/202659035</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>3552.19</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3552.19</v>
+      </c>
+      <c r="G4" t="n">
+        <v>212.19</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>PDF is 2 bars at $360 = $720, 3 bars at $360 = $1,080, and 2 bars at $770 = $1,540. Subtotal $3,340, freight $212.19, tax $0, total $3,552.19. Verification matches. KIMCO has no merchandise lines and only the $212.19 freight fee, so Invoice_Amount is $212.19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>10469</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1110-LUXOR STAFFING, INC.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2221</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>3587.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3587.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3587.5</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>10470</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1150-RYERSON, JOSEPH T. &amp; SON</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>9307057099</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>703.3099999999999</v>
+      </c>
+      <c r="F6" t="n">
+        <v>703.3099999999999</v>
+      </c>
+      <c r="G6" t="n">
+        <v>703.3099999999999</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>10471</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1043-CAPITAL MACHINE TECHNOLOGIES</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PS-INV103317</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>610</v>
+      </c>
+      <c r="F7" t="n">
+        <v>610</v>
+      </c>
+      <c r="G7" t="n">
+        <v>610</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>PDF is labor qty 2 at $210 = $420, shop supplies qty 1 at $25, and travel qty 1 at $165. Total $610, no tax, PO 58989. Verification and Invoice_Amount are $610. KIMCO receipt 25235 is qty 1 at $298.71, plus fees of $165, $25, and a second $165, and a PPV of -$43.71. The qty and the extra $165 fee do not match the PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>10475</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1135-ONEAL STEEL, LLC.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>15409416</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>42818.73</v>
+      </c>
+      <c r="F8" t="n">
+        <v>42818.73</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>The attached PDF is a 2026-09-17 payment-status letter totaling $42,818.73. It is not invoice 15409416. Verification is that letter total. There are no lines, and Invoice_Amount is $0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>10476</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1327-AM CASTLE &amp; CO</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>43293871</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>645</v>
+      </c>
+      <c r="F9" t="n">
+        <v>645</v>
+      </c>
+      <c r="G9" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PDF is 3 pieces at $215 = $645, tax $0, PO 58407, invoice total $645. Verification matches. There are no merchandise lines. Two $3.23 fees (the early-pay discount, entered twice) make Invoice_Amount $6.46.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10477</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1135-ONEAL STEEL, LLC.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>15478871</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>42079.26</v>
+      </c>
+      <c r="F10" t="n">
+        <v>42079.26</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>The attached PDF is a 2026-09-23 pending-orders letter totaling $42,079.26. It is not invoice 15478871. There are no lines, and Invoice_Amount is $0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10478</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1069-GAS AND SUPPLY</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0040455879</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>192</v>
+      </c>
+      <c r="F11" t="n">
+        <v>192</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>PDF invoice 0040455879 dated 09/28/26 is OTCL7250B04 qty 100 at $1.92 = $192.00, tax $0. Verification matches. There are no lines, so Invoice_Amount is $0. Batch 747.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10479</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1069-GAS AND SUPPLY</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0040455916</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>138.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>138.5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>PDF is 2 AR90CD300 cylinders at $28 = $56, 2 ARG300 cylinders at $30 = $60, and a fuel surcharge of $22.50. Subtotal $138.50, tax $0. Verification matches. KIMCO saved only the $22.50 fuel fee. The $116 of merchandise is missing, so Invoice_Amount is $22.50.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>10480</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1069-GAS AND SUPPLY</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>0040455615</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>213.93</v>
+      </c>
+      <c r="F13" t="n">
+        <v>213.93</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PDF invoice 0040455615, PO 59081, is MLW49-22-4170 qty 1 at $213.93, tax $0. Verification matches. There are no lines, so Invoice_Amount is $0. The second page of the file is a different invoice, 0040455291.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>10481</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1150-RYERSON, JOSEPH T. &amp; SON</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>9307115285</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>721.55</v>
+      </c>
+      <c r="F14" t="n">
+        <v>721.55</v>
+      </c>
+      <c r="G14" t="n">
+        <v>721.55</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>PDF is 12 pieces at $60 = $720 plus fuel $1.55, tax $0, total $721.55, PO 59176. KIMCO receipt 24866 is qty 84 at $8.5714 = $720 plus the $1.55 fuel fee. The totals match. The qty does not: 12 pieces versus 84.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>10482</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1157-SHOPPA'S MATERIAL HANDLING</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PSI-001239218</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>608.58</v>
+      </c>
+      <c r="F15" t="n">
+        <v>608.58</v>
+      </c>
+      <c r="G15" t="n">
+        <v>633.58</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>PDF is materials $132.20 + labor $430.00 + sales tax $46.38 = $608.58. Verification matches. KIMCO has no merchandise lines and no Taxes tab. A $608.58 fee plus an extra $25 fee (the parts-return policy note) make Invoice_Amount $633.58.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>10483</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1157-SHOPPA'S MATERIAL HANDLING</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PSI-001240544</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>806.97</v>
+      </c>
+      <c r="F16" t="n">
+        <v>806.97</v>
+      </c>
+      <c r="G16" t="n">
+        <v>831.97</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>PDF is materials $207.97 + labor $537.50 + sales tax $61.50 = $806.97. Verification matches. KIMCO has no merchandise lines and no Taxes tab. A $806.97 fee plus an extra $25 fee make Invoice_Amount $831.97.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>10484</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1181-TPI</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>18528</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1086.6</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1086.6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>PDF is 10 fenders at $108.66 = $1,086.60, PO 58897, dated 22-Sep-26. Verification matches. There are no lines, so Invoice_Amount is $0. Batch 375.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>10485</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1181-TPI</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>18529</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>6519.6</v>
+      </c>
+      <c r="F18" t="n">
+        <v>6519.6</v>
+      </c>
+      <c r="G18" t="n">
+        <v>6519.6</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>10486</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1181-TPI</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>18530</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>3259.8</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3259.8</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>PDF is 30 fenders at $108.66 = $3,259.80, PO 58931, dated 22-Sep-26. Verification matches. There are no lines, so Invoice_Amount is $0. Batch 375.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>10487</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1020-AMERICAN QUALITY POWDERCOATING</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>11044</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>520</v>
+      </c>
+      <c r="F20" t="n">
+        <v>520</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>PDF invoice 11044, PO 59171, dated 09/29/2026, is 1 at $445, two lines at $5, 3 at $10, 1 at $10, and 1 at $25, total $520. Verification matches. There are no lines, so Invoice_Amount is $0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>10488</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1020-AMERICAN QUALITY POWDERCOATING</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>11043</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>150</v>
+      </c>
+      <c r="F21" t="n">
+        <v>150</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>PDF is 5 at $30 = $150, PO 59263, dated 09/29/2026. Verification matches. There are no lines, so Invoice_Amount is $0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>10489</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1020-AMERICAN QUALITY POWDERCOATING</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>11042</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>2600</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>PDF invoice 11042, PO 59276, is 5 at $445, 5 at $5, 5 at $5, 15 at $10, 5 at $10, and 5 at $25, total $2,600. Verification matches. There are no lines, so Invoice_Amount is $0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>10490</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1020-AMERICAN QUALITY POWDERCOATING</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>11041</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>250</v>
+      </c>
+      <c r="F23" t="n">
+        <v>250</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>PDF is 250 spacers at $1 = $250, PO 59274, dated 09/28/2026. Verification matches. There are no lines, so Invoice_Amount is $0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>10491</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1181-TPI</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>18564</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>434.64</v>
+      </c>
+      <c r="F24" t="n">
+        <v>434.64</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>PDF is 4 fenders at $108.66 = $434.64, PO 58931, dated 24-Sep-26. Verification matches. There are no lines, so Invoice_Amount is $0. Batch 375.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>10492</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1337-XCALIBER</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>WB4337861639</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1080</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1080</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2160</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>PDF is 300 bearings at $3.60 = $1,080.00, tax $0, PO 59278, dated 09/27/2026, total $1,080. Verification matches. Receipt 24859 is still selected (300 at $3.60 = $1,080) and a Fees charge of $1,080 was also saved, so Invoice_Amount is $2,160. Batch 375. Not posted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>10493</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1200-WILLBANKS METALS</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>216055</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>381.72</v>
+      </c>
+      <c r="F26" t="n">
+        <v>381.72</v>
+      </c>
+      <c r="G26" t="n">
+        <v>381.72</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>PDF is 1 piece, 272.66 lb, amount $381.72, PO 59254, dated 9/29/2026, total $381.72. KIMCO receipt 25161 is qty 288 at $1.3254 with offsetting PPVs of -$1.32 and +$1.32. The total matches. The qty does not: 1 versus 288.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>10494</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1206-EMJ Earl M. Jorgensen Company</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>T609053432</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>487.14</v>
+      </c>
+      <c r="F27" t="n">
+        <v>487.14</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>PDF invoice T609053432 is 1 tube, 23.12 at $21.07 = $487.14, PO 59273, tax blank, total $487.14. Verification matches. There are no lines, so Invoice_Amount is $0. Batch 375. The second page is a different invoice, T609084432.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>10495</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1069-GAS AND SUPPLY</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>0040459813</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>66</v>
+      </c>
+      <c r="F28" t="n">
+        <v>66</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>PDF invoice 0040459813 dated 09/29/26 is WSP1801S0020 qty 12 at $5.50 = $66.00, tax $0. Verification matches. There are no lines, so Invoice_Amount is $0. Batch 747.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>10496</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1020-AMERICAN QUALITY POWDERCOATING</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>11052</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>150</v>
+      </c>
+      <c r="F29" t="n">
+        <v>150</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>PDF is 15 at $10 = $150, PO 59315, dated 09/30/2026. Verification matches. There are no lines, so Invoice_Amount is $0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>10497</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1020-AMERICAN QUALITY POWDERCOATING</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>11051</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>250</v>
+      </c>
+      <c r="F30" t="n">
+        <v>250</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>PDF is 5 at $50 = $250, PO 59312, dated 09/30/2026. Verification matches. There are no lines, so Invoice_Amount is $0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>10498</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1020-AMERICAN QUALITY POWDERCOATING</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>11050</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>500</v>
+      </c>
+      <c r="F31" t="n">
+        <v>500</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>PDF is 10 at $50 = $500, PO 59314, dated 09/30/2026. Verification matches. There are no lines, so Invoice_Amount is $0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>10499</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1020-AMERICAN QUALITY POWDERCOATING</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>11049</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>300</v>
+      </c>
+      <c r="F32" t="n">
+        <v>300</v>
+      </c>
+      <c r="G32" t="n">
+        <v>300</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>PDF is 12 at $25 = $300, PO 59281, dated 09/30/2026, total $300. Verification and Invoice_Amount are $300. KIMCO saved a $300 fee and no merchandise line for qty 12 at $25.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>10500</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1020-AMERICAN QUALITY POWDERCOATING</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>11047</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>590</v>
+      </c>
+      <c r="F33" t="n">
+        <v>590</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>PDF invoice 11047, PO 59298, is 18 at $10, 18 at $10, 10 at $18, and 1 at $50, total $590. Verification matches. There are no lines, so Invoice_Amount is $0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>10501</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1200-WILLBANKS METALS</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>216127</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>5760</v>
+      </c>
+      <c r="F34" t="n">
+        <v>5760</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>PDF is 20 pieces, 3,600 lb, amount $5,760, PO 59277, dated 9/30/2026. Verification matches. There are no lines, so Invoice_Amount is $0. Batch 375.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>10502</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1143-PRIORITY 1</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>18440283</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>219.09</v>
+      </c>
+      <c r="F35" t="n">
+        <v>219.09</v>
+      </c>
+      <c r="G35" t="n">
+        <v>219.09</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>10503</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1206-EMJ Earl M. Jorgensen Company</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>S816901432</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>166.98</v>
+      </c>
+      <c r="F36" t="n">
+        <v>166.98</v>
+      </c>
+      <c r="G36" t="n">
+        <v>166.98</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>PDF is 1 bar, 138 at $1.21 = $166.98, PO 59323, tax blank, total $166.98. KIMCO receipt 25160 is qty 240 at $0.6857 plus a PPV of $2.41. The total matches. The qty does not: 138 versus 240.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>10504</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1135-ONEAL STEEL, LLC.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>15486572</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>326.12</v>
+      </c>
+      <c r="F37" t="n">
+        <v>326.12</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>PDF invoice 15486572, PO 59200, is lines of $107.12 and $219.00, total $326.12, freight $0, tax $0. Verification matches. There are no lines, so Invoice_Amount is $0. Batch 375.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>10505</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1135-ONEAL STEEL, LLC.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>15486598</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>3012.19</v>
+      </c>
+      <c r="F38" t="n">
+        <v>3012.19</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>PDF invoice 15486598, PO 59251, is 10 pieces, line total $3,012.19, freight $0, tax $0. Verification matches. There are no lines, so Invoice_Amount is $0. Batch 375.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>10506</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1135-ONEAL STEEL, LLC.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>15486600</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>16386.88</v>
+      </c>
+      <c r="F39" t="n">
+        <v>16386.88</v>
+      </c>
+      <c r="G39" t="n">
+        <v>16386.88</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>10507</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1135-ONEAL STEEL, LLC.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>15486770</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>502.32</v>
+      </c>
+      <c r="F40" t="n">
+        <v>502.32</v>
+      </c>
+      <c r="G40" t="n">
+        <v>502.32</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>PDF invoice 15486770, PO 59279, is 4 pieces of 1-1/2 SCH 40, extended $502.32, freight $0, tax $0. KIMCO receipt 25186 is qty 1008 at $0.4984 plus a PPV of -$0.07. The total matches. The qty does not: 4 versus 1008.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>10508</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1135-ONEAL STEEL, LLC.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>15486823</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>10713.89</v>
+      </c>
+      <c r="F41" t="n">
+        <v>10713.89</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>PDF invoice 15486823, PO 59289, is line totals $4,847.12 + $4,101.93 + $1,764.84 = $10,713.89, freight $0. Verification matches. There are no lines, so Invoice_Amount is $0. Batch 375.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>10509</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1135-ONEAL STEEL, LLC.</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>15486842</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>API Agent - 10/6/26 Sept (747)</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>5328.46</v>
+      </c>
+      <c r="F42" t="n">
+        <v>5328.46</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>PDF invoice 15486842, PO 59293, is lines of $117.93, $4,015.00, $687.53, and $508.00, total $5,328.46, freight $0. Verification matches. There are no lines, so Invoice_Amount is $0. Batch 747.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H42"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>